<commit_message>
Added SOP Format, Annexure request and Issue flow.
</commit_message>
<xml_diff>
--- a/src/test/resources/testData_SOP/sop_contents.xlsx
+++ b/src/test/resources/testData_SOP/sop_contents.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="61">
   <si>
     <t xml:space="preserve">Section</t>
   </si>
@@ -198,6 +198,56 @@
   </si>
   <si>
     <t xml:space="preserve">sop.digitalSignature.dept</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sop.formatRequest.reprintReason</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF2A00FF"/>
+        <rFont val="Monospace"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Playwright</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Monospace"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF2A00FF"/>
+        <rFont val="Monospace"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">Automation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF000000"/>
+        <rFont val="Monospace"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF2A00FF"/>
+        <rFont val="Monospace"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve">purpose</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -207,11 +257,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -234,6 +285,18 @@
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="Monospace"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF2A00FF"/>
+      <name val="Monospace"/>
+      <family val="0"/>
     </font>
   </fonts>
   <fills count="2">
@@ -278,7 +341,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -291,6 +354,14 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -300,6 +371,66 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF2A00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -309,7 +440,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="10.76953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.78515625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.55"/>
   </cols>
@@ -386,8 +517,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
-  <sheetFormatPr defaultColWidth="10.76953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:B28"/>
+  <sheetFormatPr defaultColWidth="10.78515625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30.88"/>
   </cols>
@@ -606,6 +737,14 @@
       </c>
       <c r="B27" s="2" t="s">
         <v>21</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated the extent reporting to enhance report output
</commit_message>
<xml_diff>
--- a/src/test/resources/testData_SOP/sop_contents.xlsx
+++ b/src/test/resources/testData_SOP/sop_contents.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="SOP_Contents" sheetId="1" state="visible" r:id="rId2"/>
@@ -50,19 +50,22 @@
     <t xml:space="preserve">Procedure</t>
   </si>
   <si>
-    <t xml:space="preserve">Carry Out The Following Activities As Per Yearly or As &amp; When Required Schedule: The area shall be inspected by the respective user department personnel with engineering personal on yearly basis to assess the building maintenance status. The required work shall be informed to engineering department through building maintenance requisition in Format No.:EMD/030-F01 titled "Requisition of Building Maintenance". After completion of work, it shall be checked by respective user department. In addition, as part of preventive maintenance the area shall be inspected by Maintenance personnel to assess the building maintenance status. The observation will be reported in Format No.: EMD/030-F02 titled "Checklist for Building Maintenance " and on completion of the work it shall be intimated to Head Engineering and Head Q.A. Cracks or damages are noticed then arrange for repairs, ensuring no product (at any stage) is lying in the area requiring repairs, preferably during holiday or complete shutdown of the plant after covering of all the equipment by Concerned Departments. Ensure the proper removal of the rubble or building materials after completion of the repair. For any work mentioned in scope by concerned department, work permit shall be raised and approval to be taken from Engineering department, concerned department and Quality Assurance. Civil Work: Work order shall be initiated by Sr. Technician / Officer / Executive Engineer and handed over to concerned agency. The area shall be spared and equipment shall be covered by concerned department If any product or material is lying in same area, it shall be removed On completion of work, area shall be cleaned and sanitized (if required). Concerned department / Quality Assurance (wherever applicable) shall inspect area. Painting Work: Work order shall be initiated by Sr. Technician / Officer / Executive Engineer and handed over to concerned agency. Painting shall be carried out after any modification in civil work of any part of building. The area shall be spared and equipment shall be covered by concerned department.</t>
+    <t xml:space="preserve">PROCEDURE: Pre-Unloading Activities: On arrival of the vehicle at security main gate warehouse personnel shall ensure the following check point but not limited to: After arrival of vehicle at security main gate, security personnel shall inform to warehouse department and make the entry in gate inward register with stamp of gate inward on Invoice / Challan and send the loaded vehicle to material receiving area. Warehouse officer / designee shall check the physical condition of the vehicle like cleanliness, covered / closed condition i.e. shall not be exposed to outside environment and ensure the protection of the consignment. Inspect the flooring of the vehicle for the absent any oil, grease, colouring matter, spilled of material from other container, water, rusty etc. If any abnormality found while inspecting of the vehicle, inform to department Head / designee and QA Head for further actions.  Unloading &amp; Verification Activities: Check the physical condition of material and unload the material safely from the vehicle in pallets and ensure the complete unloading. After unloading the material de dust, the external surface of all the drum / bags / box / barrel etc. with the help of vacuum cleaner or lint free cloth/ duster. After de-dusting the material transfer to nearby weighing balance for verification. Warehouse personnel shall physically check the details of documents received with material as per Format No.: WHD/001-F01 titled “Checklist for Receipt of Raw Material”. Warehouse personnel shall check the correctness of documents received along with material such as invoice, challan, COA, LR copy etc. and received COA shall be readable and legible. The manufacturer label shall contain the details like Name, Batch No., Mfg. Date, Exp. Date / Retest Date, Quantity, Manufacturer name, Manufacturing site address, storage condition etc. QR code on the API manufacturer label shall be mandatory. Warehouse personnel shall scan the QR code and verify the manufacturer label details. If any API does not have a label with a QR code, warehouse personnel shall not receive that material and the material shall be returned to the supplier and same shall be informed to QA. Warehouse personnel shall check the supplier and manufacturer details of material with Approved vendor list. Address mentioned on the container label shall match with the address mentioned in Approved Vendor List. If any material received apart from approved vendor list, warehouse personnel shall not accept the material and intimation shall be given to QA Head and Purchase department through mail. Verify the quantity of materials by weighing against the invoice/ packing list and record the details as per Format No.: WHD/001-F02 titled “Weighing of Raw Material”. Note: If a barrel of solvent or liquid is received, the physical weight of the barrel shall not be verified, the gross/net weight as given by the vendor shall be recorded. If material found satisfactory the warehouse personnel shall store the material into storage area. If any specific storage condition material received e.g. 2 to 8°C, ensure the availability of data logger. Check condition of vehicle/temperature control box if any material has received a specific storage condition e.g. 2 to 8° C If the data logger is available, then press the "STOP" button on the data logger for a few seconds and stop the temperature recording. Connect the data logger to the computer system and review the data by downloading the data from the data logger. If any abnormality found in the temperature data inform to QA Head / designee and QA Head / designee shall take appropriate decision for further process. Warehouse personnel affix the received stamped on delivery challan / Invoice / LR copy and handover one copy of delivery challan / Invoice / LR copy to vehicle driver/ supplier. Handling of Damage Goods: In case of damaged container identified during the physical verification segregate the damaged pack from other packs. Check the extent of damage whether it affects to other material or not. Check the material whether it spilled or not, check the material whether it exposed to the open environment or not. Inform to warehouse Head / designee, purchase department and QA Head / designee. QA Head / designee shall take appropriate decision based upon the extent &amp; nature of damage. In case of damage in the consignment of Raw Material as explained in point no. 7.3.3, shall be sent back to the manufacturer/ supplier. Note: If barrel / drum leakage of liquid or solvent material found then the material will not be accepted.  Preparation of Goods Receipt Note (GRN): Click on link of Pharmaverge ERP  https://erp.hofpharma.com/webui/     Creator shall Login using User ID, Password and Click OK button.    After login into ERP the following screen shall appear.    Type Goods Receipt Note in Search Bar and enter.    To prepare new SOP click on (+) button.   Fill the details of GRN to be prepared, Select Organization-HOF Pharmaceuticals Ltd, Document type - RM Receipt, Date, Account Date, Businnes Partner- Name of Supplier, Warehouse, Challan No. - Invoice No.,Challan Date. To add Receipt Line for Material details, click in create lines from.    After click in create lines from the following screen shall appear.    Click in down arrow of Order and select Purchase Order No.    Tick the order line and after tick on Create liness from Shipment/ Receipt.    After click in Create liness from Shipment/ Receipt the following screen shall appear and Tick on Edit Record.    After click in Edit Record the following screen shall appear.    Fill the details of material, Quantity Invoiced, Excess Qty/ Shortage Qty (if required), No of Case, Pack Quantity, Batch No., Mfg, By, Mfg. Date, Exp. Date, Retest Date, Stoage Condition, Date Format. After fill the details of material, click on Goods Receipt Note.    After click in Goods Receipt Note the following screen shall appear and tick on Document Action.    After tick on Document Action "Complete" tick on tick mark.    Print the GRN, click on  and printout and signature it.       Prepare Material Label: Click on  and select QR Material Status Label and then tick  Button.      After click on Button, the preview of Material Label and Printout and signature it.   PrepareTest Request: Type RM/PM Sampling Request in Search Bar and click.    After click on RM/PM Sampling Request the following screen shall appear. Then enter Request Date.    Click on Document Action and Prepare it.      After click on Button, click on the following icon  and Print the "Test Request" and signature it.       Send signed copy of Test Request slip along with COA of received material to Quality Control department. Send signed copy of GRN along with Invoice / Challan to account department. Goods receipt number shall be generated using combination of alpha-numeric characters, The Goods receipt numbering system will be as per RMXXYYYY. Where; RM          : Stand for Raw Material XX           : Stand for last two digit of running calendar year YYYY      : Stand for serial no. of material receipt at site. i.e. start from 0001 so on. Serial no shall be re-start from 0001 from the 1st January of every year. Example: A typical GRN No. for Raw Material is written as “RM250001. Inward number shall be generated using combination of alpha-numeric characters, The Inward numbering system will be as per PIHPLRMXXYYYYYY. Where; PI               : Stand for Pipan Location HPL           : Stand for material of HOF Pharmaceuticals Ltd RM            : Stand for Raw Material XX             : Stand for last two digit of running calendar year YYYYYY    : Stand for serial no. of material receipt at site. i.e. start from 000001 to so on., Serial no shall be re-start from 0001 from the 1st January of every year. Note: If Expiry Date is not available in vendor COA, and only retest date available, retest date shall be considered as expiry date for received materials. Also, material shall not be used after expiry / retest given by manufacturer. Raw Material Inward Register Record: Type RM Inward Register in Search Bar and click.    After click on RM Inward Register the following screen shall appear. Then enter warehouse - RM Store and Enter Movement Date.    After fill the details click on Button and generate Inward Register.      Verification of Material Status: Open the ERP system on your Mobile / Tablet device as per Point No. 7.4.1 to 7.4.3. Type Status Label in Search Bar and click.    After click on Satus Label the following screen shall appear. Then click on barcode scanner.    After click on the barcode scanner and then scan the barcode on the material label. The status of the Material shall appear as per the following screen,                                             
+Carry Out The Following Activities As Per Yearly or As &amp; When Required Schedule: The area shall be inspected by the respective user department personnel with engineering personal on yearly basis to assess the building maintenance status. The required work shall be informed to engineering department through building maintenance requisition in Format No.:EMD/030-F01 titled "Requisition of Building Maintenance". After completion of work, it shall be checked by respective user department. In addition, as part of preventive maintenance the area shall be inspected by Maintenance personnel to assess the building maintenance status. The observation will be reported in Format No.: EMD/030-F02 titled "Checklist for Building Maintenance " and on completion of the work it shall be intimated to Head Engineering and Head Q.A. Cracks or damages are noticed then arrange for repairs, ensuring no product (at any stage) is lying in the area requiring repairs, preferably during holiday or complete shutdown of the plant after covering of all the equipment by Concerned Departments. Ensure the proper removal of the rubble or building materials after completion of the repair. For any work mentioned in scope by concerned department, work permit shall be raised and approval to be taken from Engineering department, concerned department and Quality Assurance. Civil Work: Work order shall be initiated by Sr. Technician / Officer / Executive Engineer and handed over to concerned agency. The area shall be spared and equipment shall be covered by concerned department If any product or material is lying in same area, it shall be removed On completion of work, area shall be cleaned and sanitized (if required). Concerned department / Quality Assurance (wherever applicable) shall inspect area. Painting Work: Work order shall be initiated by Sr. Technician / Officer / Executive Engineer and handed over to concerned agency. Painting shall be carried out after any modification in civil work of any part of building. The area shall be spared and equipment shall be covered by concerned department.</t>
   </si>
   <si>
     <t xml:space="preserve">AnnexureContent</t>
   </si>
   <si>
-    <t xml:space="preserve">YEAR :- ___________ SR NO CHECKLIST SCHEDULE JAN FEB MAR APR MAY JUN JULY AUG SEP OCT NOV DEC 1 Facility Room Checklist PLANNED Q Q Q Q ACTUAL 2 Paint Record PLANNED H H ACTUAL 3 Roof Leak Check Record PLANNED H H ACTUAL 4 Crack Inspection Record PLANNED H H ACTUAL 5 Epoxy / Kota Flooring Inspection Record PLANNED H H ACTUAL</t>
+    <t xml:space="preserve">YEAR :- ___________ SR NO CHECKLIST SCHEDULE JAN FEB MAR APR MAY JUN JULY AUG SEP OCT NOV DEC 1 Facility Room Checklist PLANNED Q Q Q Q ACTUAL 2 Paint Record PLANNED H H ACTUAL 3 Roof Leak Check Record PLANNED H H ACTUAL 4 Crack Inspection Record PLANNED H H ACTUAL 5 Epoxy / Kota Flooring Inspection Record PLANNED H H ACTUAL
+PROCEDURE: Pre-Unloading Activities: On arrival of the vehicle at security main gate warehouse personnel shall ensure the following check point but not limited to: After arrival of vehicle at security main gate, security personnel shall inform to warehouse department and make the entry in gate inward register with stamp of gate inward on Invoice / Challan and send the loaded vehicle to material receiving area. Warehouse officer / designee shall check the physical condition of the vehicle like cleanliness, covered / closed condition i.e. shall not be exposed to outside environment and ensure the protection of the consignment. Inspect the flooring of the vehicle for the absent any oil, grease, colouring matter, spilled of material from other container, water, rusty etc. If any abnormality found while inspecting of the vehicle, inform to department Head / designee and QA Head for further actions.  Unloading &amp; Verification Activities: Check the physical condition of material and unload the material safely from the vehicle in pallets and ensure the complete unloading. After unloading the material de dust, the external surface of all the drum / bags / box / barrel etc. with the help of vacuum cleaner or lint free cloth/ duster. After de-dusting the material transfer to nearby weighing balance for verification. Warehouse personnel shall physically check the details of documents received with material as per Format No.: WHD/001-F01 titled “Checklist for Receipt of Raw Material”. Warehouse personnel shall check the correctness of documents received along with material such as invoice, challan, COA, LR copy etc. and received COA shall be readable and legible. The manufacturer label shall contain the details like Name, Batch No., Mfg. Date, Exp. Date / Retest Date, Quantity, Manufacturer name, Manufacturing site address, storage condition etc. QR code on the API manufacturer label shall be mandatory. Warehouse personnel shall scan the QR code and verify the manufacturer label details. If any API does not have a label with a QR code, warehouse personnel shall not receive that material and the material shall be returned to the supplier and same shall be informed to QA. Warehouse personnel shall check the supplier and manufacturer details of material with Approved vendor list. Address mentioned on the container label shall match with the address mentioned in Approved Vendor List. If any material received apart from approved vendor list, warehouse personnel shall not accept the material and intimation shall be given to QA Head and Purchase department through mail. Verify the quantity of materials by weighing against the invoice/ packing list and record the details as per Format No.: WHD/001-F02 titled “Weighing of Raw Material”. Note: If a barrel of solvent or liquid is received, the physical weight of the barrel shall not be verified, the gross/net weight as given by the vendor shall be recorded. If material found satisfactory the warehouse personnel shall store the material into storage area. If any specific storage condition material received e.g. 2 to 8°C, ensure the availability of data logger. Check condition of vehicle/temperature control box if any material has received a specific storage condition e.g. 2 to 8° C If the data logger is available, then press the "STOP" button on the data logger for a few seconds and stop the temperature recording. Connect the data logger to the computer system and review the data by downloading the data from the data logger. If any abnormality found in the temperature data inform to QA Head / designee and QA Head / designee shall take appropriate decision for further process. Warehouse personnel affix the received stamped on delivery challan / Invoice / LR copy and handover one copy of delivery challan / Invoice / LR copy to vehicle driver/ supplier. Handling of Damage Goods: In case of damaged container identified during the physical verification segregate the damaged pack from other packs. Check the extent of damage whether it affects to other material or not. Check the material whether it spilled or not, check the material whether it exposed to the open environment or not. Inform to warehouse Head / designee, purchase department and QA Head / designee. QA Head / designee shall take appropriate decision based upon the extent &amp; nature of damage. In case of damage in the consignment of Raw Material as explained in point no. 7.3.3, shall be sent back to the manufacturer/ supplier. Note: If barrel / drum leakage of liquid or solvent material found then the material will not be accepted.  Preparation of Goods Receipt Note (GRN): Click on link of Pharmaverge ERP  https://erp.hofpharma.com/webui/     Creator shall Login using User ID, Password and Click OK button.    After login into ERP the following screen shall appear.    Type Goods Receipt Note in Search Bar and enter.    To prepare new SOP click on (+) button.   Fill the details of GRN to be prepared, Select Organization-HOF Pharmaceuticals Ltd, Document type - RM Receipt, Date, Account Date, Businnes Partner- Name of Supplier, Warehouse, Challan No. - Invoice No.,Challan Date. To add Receipt Line for Material details, click in create lines from.    After click in create lines from the following screen shall appear.    Click in down arrow of Order and select Purchase Order No.    Tick the order line and after tick on Create liness from Shipment/ Receipt.    After click in Create liness from Shipment/ Receipt the following screen shall appear and Tick on Edit Record.    After click in Edit Record the following screen shall appear.    Fill the details of material, Quantity Invoiced, Excess Qty/ Shortage Qty (if required), No of Case, Pack Quantity, Batch No., Mfg, By, Mfg. Date, Exp. Date, Retest Date, Stoage Condition, Date Format. After fill the details of material, click on Goods Receipt Note.    After click in Goods Receipt Note the following screen shall appear and tick on Document Action.    After tick on Document Action "Complete" tick on tick mark.    Print the GRN, click on  and printout and signature it.       Prepare Material Label: Click on  and select QR Material Status Label and then tick  Button.      After click on Button, the preview of Material Label and Printout and signature it.   PrepareTest Request: Type RM/PM Sampling Request in Search Bar and click.    After click on RM/PM Sampling Request the following screen shall appear. Then enter Request Date.    Click on Document Action and Prepare it.      After click on Button, click on the following icon  and Print the "Test Request" and signature it.       Send signed copy of Test Request slip along with COA of received material to Quality Control department. Send signed copy of GRN along with Invoice / Challan to account department. Goods receipt number shall be generated using combination of alpha-numeric characters, The Goods receipt numbering system will be as per RMXXYYYY. Where; RM          : Stand for Raw Material XX           : Stand for last two digit of running calendar year YYYY      : Stand for serial no. of material receipt at site. i.e. start from 0001 so on. Serial no shall be re-start from 0001 from the 1st January of every year. Example: A typical GRN No. for Raw Material is written as “RM250001. Inward number shall be generated using combination of alpha-numeric characters, The Inward numbering system will be as per PIHPLRMXXYYYYYY. Where; PI               : Stand for Pipan Location HPL           : Stand for material of HOF Pharmaceuticals Ltd RM            : Stand for Raw Material XX             : Stand for last two digit of running calendar year YYYYYY    : Stand for serial no. of material receipt at site. i.e. start from 000001 to so on., Serial no shall be re-start from 0001 from the 1st January of every year. Note: If Expiry Date is not available in vendor COA, and only retest date available, retest date shall be considered as expiry date for received materials. Also, material shall not be used after expiry / retest given by manufacturer. Raw Material Inward Register Record: Type RM Inward Register in Search Bar and click.    After click on RM Inward Register the following screen shall appear. Then enter warehouse - RM Store and Enter Movement Date.    After fill the details click on Button and generate Inward Register.      Verification of Material Status: Open the ERP system on your Mobile / Tablet device as per Point No. 7.4.1 to 7.4.3. Type Status Label in Search Bar and click.    After click on Satus Label the following screen shall appear. Then click on barcode scanner.    After click on the barcode scanner and then scan the barcode on the material label. The status of the Material shall appear as per the following screen,                                             </t>
   </si>
   <si>
     <t xml:space="preserve">FormatContent</t>
   </si>
   <si>
-    <t xml:space="preserve">SR NO. Name of the Area Type of paint Paint Done on Checked by(Sign/Date) Remark</t>
+    <t xml:space="preserve">SR NO. Name of the Area Type of paint Paint Done on Checked by(Sign/Date) Remark
+PROCEDURE: Pre-Unloading Activities: On arrival of the vehicle at security main gate warehouse personnel shall ensure the following check point but not limited to: After arrival of vehicle at security main gate, security personnel shall inform to warehouse department and make the entry in gate inward register with stamp of gate inward on Invoice / Challan and send the loaded vehicle to material receiving area. Warehouse officer / designee shall check the physical condition of the vehicle like cleanliness, covered / closed condition i.e. shall not be exposed to outside environment and ensure the protection of the consignment. Inspect the flooring of the vehicle for the absent any oil, grease, colouring matter, spilled of material from other container, water, rusty etc. If any abnormality found while inspecting of the vehicle, inform to department Head / designee and QA Head for further actions.  Unloading &amp; Verification Activities: Check the physical condition of material and unload the material safely from the vehicle in pallets and ensure the complete unloading. After unloading the material de dust, the external surface of all the drum / bags / box / barrel etc. with the help of vacuum cleaner or lint free cloth/ duster. After de-dusting the material transfer to nearby weighing balance for verification. Warehouse personnel shall physically check the details of documents received with material as per Format No.: WHD/001-F01 titled “Checklist for Receipt of Raw Material”. Warehouse personnel shall check the correctness of documents received along with material such as invoice, challan, COA, LR copy etc. and received COA shall be readable and legible. The manufacturer label shall contain the details like Name, Batch No., Mfg. Date, Exp. Date / Retest Date, Quantity, Manufacturer name, Manufacturing site address, storage condition etc. QR code on the API manufacturer label shall be mandatory. Warehouse personnel shall scan the QR code and verify the manufacturer label details. If any API does not have a label with a QR code, warehouse personnel shall not receive that material and the material shall be returned to the supplier and same shall be informed to QA. Warehouse personnel shall check the supplier and manufacturer details of material with Approved vendor list. Address mentioned on the container label shall match with the address mentioned in Approved Vendor List. If any material received apart from approved vendor list, warehouse personnel shall not accept the material and intimation shall be given to QA Head and Purchase department through mail. Verify the quantity of materials by weighing against the invoice/ packing list and record the details as per Format No.: WHD/001-F02 titled “Weighing of Raw Material”. Note: If a barrel of solvent or liquid is received, the physical weight of the barrel shall not be verified, the gross/net weight as given by the vendor shall be recorded. If material found satisfactory the warehouse personnel shall store the material into storage area. If any specific storage condition material received e.g. 2 to 8°C, ensure the availability of data logger. Check condition of vehicle/temperature control box if any material has received a specific storage condition e.g. 2 to 8° C If the data logger is available, then press the "STOP" button on the data logger for a few seconds and stop the temperature recording. Connect the data logger to the computer system and review the data by downloading the data from the data logger. If any abnormality found in the temperature data inform to QA Head / designee and QA Head / designee shall take appropriate decision for further process. Warehouse personnel affix the received stamped on delivery challan / Invoice / LR copy and handover one copy of delivery challan / Invoice / LR copy to vehicle driver/ supplier. Handling of Damage Goods: In case of damaged container identified during the physical verification segregate the damaged pack from other packs. Check the extent of damage whether it affects to other material or not. Check the material whether it spilled or not, check the material whether it exposed to the open environment or not. Inform to warehouse Head / designee, purchase department and QA Head / designee. QA Head / designee shall take appropriate decision based upon the extent &amp; nature of damage. In case of damage in the consignment of Raw Material as explained in point no. 7.3.3, shall be sent back to the manufacturer/ supplier. Note: If barrel / drum leakage of liquid or solvent material found then the material will not be accepted.  Preparation of Goods Receipt Note (GRN): Click on link of Pharmaverge ERP  https://erp.hofpharma.com/webui/     Creator shall Login using User ID, Password and Click OK button.    After login into ERP the following screen shall appear.    Type Goods Receipt Note in Search Bar and enter.    To prepare new SOP click on (+) button.   Fill the details of GRN to be prepared, Select Organization-HOF Pharmaceuticals Ltd, Document type - RM Receipt, Date, Account Date, Businnes Partner- Name of Supplier, Warehouse, Challan No. - Invoice No.,Challan Date. To add Receipt Line for Material details, click in create lines from.    After click in create lines from the following screen shall appear.    Click in down arrow of Order and select Purchase Order No.    Tick the order line and after tick on Create liness from Shipment/ Receipt.    After click in Create liness from Shipment/ Receipt the following screen shall appear and Tick on Edit Record.    After click in Edit Record the following screen shall appear.    Fill the details of material, Quantity Invoiced, Excess Qty/ Shortage Qty (if required), No of Case, Pack Quantity, Batch No., Mfg, By, Mfg. Date, Exp. Date, Retest Date, Stoage Condition, Date Format. After fill the details of material, click on Goods Receipt Note.    After click in Goods Receipt Note the following screen shall appear and tick on Document Action.    After tick on Document Action "Complete" tick on tick mark.    Print the GRN, click on  and printout and signature it.       Prepare Material Label: Click on  and select QR Material Status Label and then tick  Button.      After click on Button, the preview of Material Label and Printout and signature it.   PrepareTest Request: Type RM/PM Sampling Request in Search Bar and click.    After click on RM/PM Sampling Request the following screen shall appear. Then enter Request Date.    Click on Document Action and Prepare it.      After click on Button, click on the following icon  and Print the "Test Request" and signature it.       Send signed copy of Test Request slip along with COA of received material to Quality Control department. Send signed copy of GRN along with Invoice / Challan to account department. Goods receipt number shall be generated using combination of alpha-numeric characters, The Goods receipt numbering system will be as per RMXXYYYY. Where; RM          : Stand for Raw Material XX           : Stand for last two digit of running calendar year YYYY      : Stand for serial no. of material receipt at site. i.e. start from 0001 so on. Serial no shall be re-start from 0001 from the 1st January of every year. Example: A typical GRN No. for Raw Material is written as “RM250001. Inward number shall be generated using combination of alpha-numeric characters, The Inward numbering system will be as per PIHPLRMXXYYYYYY. Where; PI               : Stand for Pipan Location HPL           : Stand for material of HOF Pharmaceuticals Ltd RM            : Stand for Raw Material XX             : Stand for last two digit of running calendar year YYYYYY    : Stand for serial no. of material receipt at site. i.e. start from 000001 to so on., Serial no shall be re-start from 0001 from the 1st January of every year. Note: If Expiry Date is not available in vendor COA, and only retest date available, retest date shall be considered as expiry date for received materials. Also, material shall not be used after expiry / retest given by manufacturer. Raw Material Inward Register Record: Type RM Inward Register in Search Bar and click.    After click on RM Inward Register the following screen shall appear. Then enter warehouse - RM Store and Enter Movement Date.    After fill the details click on Button and generate Inward Register.      Verification of Material Status: Open the ERP system on your Mobile / Tablet device as per Point No. 7.4.1 to 7.4.3. Type Status Label in Search Bar and click.    After click on Satus Label the following screen shall appear. Then click on barcode scanner.    After click on the barcode scanner and then scan the barcode on the material label. The status of the Material shall appear as per the following screen,                                             </t>
   </si>
   <si>
     <t xml:space="preserve">Key</t>
@@ -209,6 +212,7 @@
         <color rgb="FF2A00FF"/>
         <rFont val="Monospace"/>
         <family val="0"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Playwright</t>
     </r>
@@ -218,6 +222,7 @@
         <color rgb="FF000000"/>
         <rFont val="Monospace"/>
         <family val="0"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> </t>
     </r>
@@ -227,6 +232,7 @@
         <color rgb="FF2A00FF"/>
         <rFont val="Monospace"/>
         <family val="0"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">Automation</t>
     </r>
@@ -236,6 +242,7 @@
         <color rgb="FF000000"/>
         <rFont val="Monospace"/>
         <family val="0"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve"> </t>
     </r>
@@ -245,6 +252,7 @@
         <color rgb="FF2A00FF"/>
         <rFont val="Monospace"/>
         <family val="0"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">purpose</t>
     </r>
@@ -291,12 +299,14 @@
       <color rgb="FF000000"/>
       <name val="Monospace"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="8"/>
       <color rgb="FF2A00FF"/>
       <name val="Monospace"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -341,7 +351,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -352,6 +362,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -440,7 +454,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="10.78515625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.55"/>
   </cols>
@@ -477,27 +491,27 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>13</v>
       </c>
     </row>
@@ -518,7 +532,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B28"/>
-  <sheetFormatPr defaultColWidth="10.78515625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30.88"/>
   </cols>
@@ -740,10 +754,10 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3" t="s">
+      <c r="A28" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="5" t="s">
         <v>60</v>
       </c>
     </row>

</xml_diff>